<commit_message>
added dataset csv file (for preview)
</commit_message>
<xml_diff>
--- a/Excel-basic-function-practice.xlsx
+++ b/Excel-basic-function-practice.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mjahn\GitHubProjects\Data-Analyst\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mjahn\GitHubProjects\Data-Analyst\day1\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{48ECB687-F825-446C-A200-62360C3B9376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -469,26 +469,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -497,42 +493,42 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf/>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -857,62 +853,34 @@
   </cols>
   <sheetData>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="23" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="25">
         <f>I9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="21" t="s">
+      <c r="G9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-      <c r="Q9" s="16"/>
-      <c r="R9" s="16"/>
-      <c r="S9" s="16"/>
-      <c r="T9" s="16"/>
-      <c r="U9" s="16"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="E10" s="30" t="s">
+      <c r="E10" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="27">
         <f>VLOOKUP(E10,DATA!$C$17:$F$26,2,FALSE)</f>
         <v>2000</v>
       </c>
-      <c r="G10" s="21"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="16"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="16"/>
-      <c r="S10" s="16"/>
-      <c r="T10" s="16"/>
-      <c r="U10" s="16"/>
+      <c r="G10" s="19"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="E11" s="6" t="s">
@@ -922,69 +890,23 @@
         <f>VLOOKUP(E11,DATA!$C$17:$F$26,2,FALSE)</f>
         <v>3000</v>
       </c>
-      <c r="G11" s="39" t="s">
+      <c r="G11" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="16"/>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="16"/>
-      <c r="S11" s="16"/>
-      <c r="T11" s="16"/>
-      <c r="U11" s="16"/>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16"/>
-      <c r="O12" s="16"/>
-      <c r="P12" s="16"/>
-      <c r="Q12" s="16"/>
-      <c r="R12" s="16"/>
-      <c r="S12" s="16"/>
-      <c r="T12" s="16"/>
-      <c r="U12" s="16"/>
-    </row>
-    <row r="13" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="16"/>
-      <c r="O13" s="16"/>
-      <c r="P13" s="16"/>
-      <c r="Q13" s="16"/>
-      <c r="R13" s="16"/>
-      <c r="S13" s="16"/>
-      <c r="T13" s="16"/>
-      <c r="U13" s="16"/>
-    </row>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
+      <c r="K11" s="36"/>
+    </row>
+    <row r="13" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="14" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="14"/>
-      <c r="R14" s="16"/>
-      <c r="S14" s="16"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="13"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
@@ -994,481 +916,438 @@
       <c r="Z14" s="1"/>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="26" t="s">
+      <c r="K15" s="14"/>
+      <c r="L15" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="M15" s="32" t="s">
+      <c r="M15" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="N15" s="32" t="s">
+      <c r="N15" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="O15" s="32" t="s">
+      <c r="O15" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="P15" s="27" t="s">
+      <c r="P15" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="Q15" s="17"/>
-      <c r="R15" s="16"/>
-      <c r="S15" s="16"/>
+      <c r="Q15" s="15"/>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="32" t="s">
+      <c r="C16" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="32" t="s">
+      <c r="E16" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="F16" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="G16" s="35" t="s">
+      <c r="G16" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="28" t="s">
+      <c r="H16" s="21"/>
+      <c r="I16" s="21"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="M16" s="33" t="s">
+      <c r="M16" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="N16" s="33" t="s">
+      <c r="N16" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="O16" s="33">
+      <c r="O16" s="29">
         <v>12000</v>
       </c>
-      <c r="P16" s="29">
+      <c r="P16" s="25">
         <v>5</v>
       </c>
-      <c r="Q16" s="17"/>
-      <c r="R16" s="16"/>
-      <c r="S16" s="16"/>
+      <c r="Q16" s="15"/>
       <c r="W16" s="2"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="29">
         <f>E17/F17</f>
         <v>2400</v>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="29">
         <v>12000</v>
       </c>
-      <c r="F17" s="33">
+      <c r="F17" s="29">
         <v>5</v>
       </c>
-      <c r="G17" s="36" t="str">
+      <c r="G17" s="32" t="str">
         <f>IF(DATA!$E17&gt;=9000,"HIGH","LOW")</f>
         <v>HIGH</v>
       </c>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="30" t="s">
+      <c r="H17" s="21"/>
+      <c r="I17" s="21"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="M17" s="34" t="s">
+      <c r="M17" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="N17" s="34" t="s">
+      <c r="N17" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="O17" s="34">
+      <c r="O17" s="30">
         <v>8000</v>
       </c>
-      <c r="P17" s="31">
+      <c r="P17" s="27">
         <v>4</v>
       </c>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="16"/>
-      <c r="S17" s="16"/>
+      <c r="Q17" s="15"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="37">
+      <c r="D18" s="33">
         <f t="shared" ref="D18:D26" si="0">E18/F18</f>
         <v>2000</v>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="30">
         <v>8000</v>
       </c>
-      <c r="F18" s="34">
+      <c r="F18" s="30">
         <v>4</v>
       </c>
-      <c r="G18" s="38" t="str">
+      <c r="G18" s="34" t="str">
         <f>IF(DATA!$E18&gt;=9000,"HIGH","LOW")</f>
         <v>LOW</v>
       </c>
-      <c r="H18" s="25" t="s">
+      <c r="H18" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="25"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="28" t="s">
+      <c r="I18" s="37"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="M18" s="33" t="s">
+      <c r="M18" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="N18" s="33" t="s">
+      <c r="N18" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="O18" s="33">
+      <c r="O18" s="29">
         <v>6000</v>
       </c>
-      <c r="P18" s="29">
+      <c r="P18" s="25">
         <v>2</v>
       </c>
-      <c r="Q18" s="17"/>
-      <c r="R18" s="16"/>
-      <c r="S18" s="16"/>
+      <c r="Q18" s="15"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="33">
+      <c r="D19" s="29">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="E19" s="33">
+      <c r="E19" s="29">
         <v>6000</v>
       </c>
-      <c r="F19" s="33">
+      <c r="F19" s="29">
         <v>2</v>
       </c>
-      <c r="G19" s="36" t="str">
+      <c r="G19" s="32" t="str">
         <f>IF(DATA!$E19&gt;=9000,"HIGH","LOW")</f>
         <v>LOW</v>
       </c>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="30" t="s">
+      <c r="H19" s="37"/>
+      <c r="I19" s="37"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="M19" s="34" t="s">
+      <c r="M19" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="N19" s="34" t="s">
+      <c r="N19" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="O19" s="34">
+      <c r="O19" s="30">
         <v>15000</v>
       </c>
-      <c r="P19" s="31">
+      <c r="P19" s="27">
         <v>6</v>
       </c>
-      <c r="Q19" s="17"/>
-      <c r="R19" s="16"/>
-      <c r="S19" s="16"/>
+      <c r="Q19" s="15"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="30">
         <f t="shared" si="0"/>
         <v>2500</v>
       </c>
-      <c r="E20" s="34">
+      <c r="E20" s="30">
         <v>15000</v>
       </c>
-      <c r="F20" s="34">
+      <c r="F20" s="30">
         <v>6</v>
       </c>
-      <c r="G20" s="38" t="str">
+      <c r="G20" s="34" t="str">
         <f>IF(DATA!$E20&gt;=9000,"HIGH","LOW")</f>
         <v>HIGH</v>
       </c>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="28" t="s">
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="M20" s="33" t="s">
+      <c r="M20" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="N20" s="33" t="s">
+      <c r="N20" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="O20" s="33">
+      <c r="O20" s="29">
         <v>7000</v>
       </c>
-      <c r="P20" s="29">
+      <c r="P20" s="25">
         <v>2</v>
       </c>
-      <c r="Q20" s="17"/>
-      <c r="R20" s="16"/>
-      <c r="S20" s="16"/>
+      <c r="Q20" s="15"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="33" t="s">
+      <c r="B21" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="33">
+      <c r="D21" s="29">
         <f t="shared" si="0"/>
         <v>3500</v>
       </c>
-      <c r="E21" s="33">
+      <c r="E21" s="29">
         <v>7000</v>
       </c>
-      <c r="F21" s="33">
+      <c r="F21" s="29">
         <v>2</v>
       </c>
-      <c r="G21" s="36" t="str">
+      <c r="G21" s="32" t="str">
         <f>IF(DATA!$E21&gt;=9000,"HIGH","LOW")</f>
         <v>LOW</v>
       </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="30" t="s">
+      <c r="K21" s="14"/>
+      <c r="L21" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="M21" s="34" t="s">
+      <c r="M21" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="N21" s="34" t="s">
+      <c r="N21" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="O21" s="34">
+      <c r="O21" s="30">
         <v>4000</v>
       </c>
-      <c r="P21" s="31">
+      <c r="P21" s="27">
         <v>1</v>
       </c>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="16"/>
-      <c r="S21" s="16"/>
+      <c r="Q21" s="15"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A22" s="30" t="s">
+      <c r="A22" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="34" t="s">
+      <c r="B22" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="34">
+      <c r="D22" s="30">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
-      <c r="E22" s="34">
+      <c r="E22" s="30">
         <v>4000</v>
       </c>
-      <c r="F22" s="34">
+      <c r="F22" s="30">
         <v>1</v>
       </c>
-      <c r="G22" s="38" t="str">
+      <c r="G22" s="34" t="str">
         <f>IF(DATA!$E22&gt;=9000,"HIGH","LOW")</f>
         <v>LOW</v>
       </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="28" t="s">
+      <c r="K22" s="14"/>
+      <c r="L22" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="M22" s="33" t="s">
+      <c r="M22" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="N22" s="33" t="s">
+      <c r="N22" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="O22" s="33">
+      <c r="O22" s="29">
         <v>11000</v>
       </c>
-      <c r="P22" s="29">
+      <c r="P22" s="25">
         <v>4</v>
       </c>
-      <c r="Q22" s="17"/>
-      <c r="R22" s="16"/>
-      <c r="S22" s="16"/>
+      <c r="Q22" s="15"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="33" t="s">
+      <c r="B23" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C23" s="33" t="s">
+      <c r="C23" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="33">
+      <c r="D23" s="29">
         <f t="shared" si="0"/>
         <v>2750</v>
       </c>
-      <c r="E23" s="33">
+      <c r="E23" s="29">
         <v>11000</v>
       </c>
-      <c r="F23" s="33">
+      <c r="F23" s="29">
         <v>4</v>
       </c>
-      <c r="G23" s="36" t="str">
+      <c r="G23" s="32" t="str">
         <f>IF(DATA!$E23&gt;=9000,"HIGH","LOW")</f>
         <v>HIGH</v>
       </c>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="30" t="s">
+      <c r="K23" s="14"/>
+      <c r="L23" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="M23" s="34" t="s">
+      <c r="M23" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="N23" s="34" t="s">
+      <c r="N23" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="O23" s="34">
+      <c r="O23" s="30">
         <v>9000</v>
       </c>
-      <c r="P23" s="31">
+      <c r="P23" s="27">
         <v>3</v>
       </c>
-      <c r="Q23" s="17"/>
-      <c r="R23" s="16"/>
-      <c r="S23" s="16"/>
+      <c r="Q23" s="15"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A24" s="30" t="s">
+      <c r="A24" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="34">
+      <c r="D24" s="30">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="E24" s="34">
+      <c r="E24" s="30">
         <v>9000</v>
       </c>
-      <c r="F24" s="34">
+      <c r="F24" s="30">
         <v>3</v>
       </c>
-      <c r="G24" s="38" t="str">
+      <c r="G24" s="34" t="str">
         <f>IF(DATA!$E24&gt;=9000,"HIGH","LOW")</f>
         <v>HIGH</v>
       </c>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="28" t="s">
+      <c r="K24" s="14"/>
+      <c r="L24" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="M24" s="33" t="s">
+      <c r="M24" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="N24" s="33" t="s">
+      <c r="N24" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="O24" s="33">
+      <c r="O24" s="29">
         <v>5000</v>
       </c>
-      <c r="P24" s="29">
+      <c r="P24" s="25">
         <v>2</v>
       </c>
-      <c r="Q24" s="17"/>
-      <c r="R24" s="16"/>
-      <c r="S24" s="16"/>
+      <c r="Q24" s="15"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="33" t="s">
+      <c r="B25" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="C25" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="29">
         <f t="shared" si="0"/>
         <v>2500</v>
       </c>
-      <c r="E25" s="33">
+      <c r="E25" s="29">
         <v>5000</v>
       </c>
-      <c r="F25" s="33">
+      <c r="F25" s="29">
         <v>2</v>
       </c>
-      <c r="G25" s="36" t="str">
+      <c r="G25" s="32" t="str">
         <f>IF(DATA!$E25&gt;=9000,"HIGH","LOW")</f>
         <v>LOW</v>
       </c>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="15"/>
+      <c r="K25" s="14"/>
       <c r="L25" s="3" t="s">
         <v>21</v>
       </c>
@@ -1484,46 +1363,39 @@
       <c r="P25" s="5">
         <v>5</v>
       </c>
-      <c r="Q25" s="17"/>
-      <c r="R25" s="16"/>
-      <c r="S25" s="16"/>
+      <c r="Q25" s="15"/>
     </row>
     <row r="26" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="34" t="s">
+      <c r="B26" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="D26" s="34">
+      <c r="D26" s="30">
         <f t="shared" si="0"/>
         <v>2600</v>
       </c>
-      <c r="E26" s="34">
+      <c r="E26" s="30">
         <v>13000</v>
       </c>
-      <c r="F26" s="34">
+      <c r="F26" s="30">
         <v>5</v>
       </c>
-      <c r="G26" s="38" t="str">
+      <c r="G26" s="34" t="str">
         <f>IF(DATA!$E26&gt;=9000,"HIGH","LOW")</f>
         <v>HIGH</v>
       </c>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="16"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="22"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="19"/>
-      <c r="O26" s="22"/>
-      <c r="P26" s="22"/>
-      <c r="Q26" s="20"/>
-      <c r="R26" s="16"/>
-      <c r="S26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="20"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="20"/>
+      <c r="P26" s="20"/>
+      <c r="Q26" s="18"/>
       <c r="T26" s="1"/>
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
@@ -1547,20 +1419,6 @@
         <v>34</v>
       </c>
       <c r="G27" s="9"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="16"/>
-      <c r="O27" s="16"/>
-      <c r="P27" s="16"/>
-      <c r="Q27" s="16"/>
-      <c r="R27" s="16"/>
-      <c r="S27" s="16"/>
-      <c r="T27" s="16"/>
-      <c r="U27" s="16"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -1574,204 +1432,114 @@
         <f>AVERAGE(DATA!$E$17:$E$26)</f>
         <v>9000</v>
       </c>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="16"/>
-      <c r="O28" s="16"/>
-      <c r="P28" s="16"/>
-      <c r="Q28" s="16"/>
-      <c r="R28" s="16"/>
-      <c r="S28" s="16"/>
-      <c r="T28" s="16"/>
-      <c r="U28" s="16"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="16"/>
-      <c r="O29" s="16"/>
-      <c r="P29" s="16"/>
-      <c r="Q29" s="16"/>
-      <c r="R29" s="16"/>
-      <c r="S29" s="16"/>
-      <c r="T29" s="16"/>
-      <c r="U29" s="16"/>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="16"/>
-      <c r="O30" s="16"/>
-      <c r="P30" s="16"/>
-      <c r="Q30" s="16"/>
-      <c r="R30" s="16"/>
-      <c r="S30" s="16"/>
-      <c r="T30" s="16"/>
-      <c r="U30" s="16"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="36"/>
+      <c r="E30" s="36"/>
+      <c r="F30" s="36"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16"/>
-      <c r="O31" s="16"/>
-      <c r="P31" s="16"/>
-      <c r="Q31" s="16"/>
-      <c r="R31" s="16"/>
-      <c r="S31" s="16"/>
-      <c r="T31" s="16"/>
-      <c r="U31" s="16"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="36"/>
+      <c r="F31" s="36"/>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="H32" s="25" t="s">
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="36"/>
+      <c r="H32" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="I32" s="25"/>
-      <c r="K32" s="25" t="s">
+      <c r="I32" s="37"/>
+      <c r="K32" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="L32" s="25"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="25" t="s">
+      <c r="L32" s="37"/>
+      <c r="N32" s="37" t="s">
         <v>40</v>
       </c>
-      <c r="O32" s="25"/>
-      <c r="P32" s="25"/>
-      <c r="Q32" s="16"/>
-      <c r="R32" s="16"/>
-      <c r="S32" s="16"/>
-      <c r="T32" s="16"/>
-      <c r="U32" s="16"/>
-    </row>
-    <row r="33" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="16"/>
-      <c r="P33" s="16"/>
-      <c r="Q33" s="16"/>
-      <c r="R33" s="16"/>
-      <c r="S33" s="16"/>
-      <c r="T33" s="16"/>
-      <c r="U33" s="16"/>
-    </row>
-    <row r="34" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="H34" s="26" t="s">
+      <c r="O32" s="37"/>
+      <c r="P32" s="37"/>
+    </row>
+    <row r="33" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="K33" s="37"/>
+      <c r="L33" s="37"/>
+    </row>
+    <row r="34" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="H34" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="I34" s="27" t="s">
+      <c r="I34" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="J34" s="16"/>
-      <c r="K34" s="26" t="s">
+      <c r="K34" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="L34" s="27" t="s">
+      <c r="L34" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M34" s="16"/>
-      <c r="N34" s="26" t="s">
+      <c r="N34" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="O34" s="32" t="s">
+      <c r="O34" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="P34" s="27" t="s">
+      <c r="P34" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="Q34" s="16"/>
-      <c r="R34" s="16"/>
-      <c r="S34" s="16"/>
-      <c r="T34" s="16"/>
-      <c r="U34" s="16"/>
-    </row>
-    <row r="35" spans="2:21" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G35">
         <v>51000</v>
       </c>
-      <c r="H35" s="28" t="s">
+      <c r="H35" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I35" s="29">
+      <c r="I35" s="25">
         <f ca="1">SUMIF(DATA!$C$17:$E$26,C17,DATA!$E$17:$E$26)</f>
         <v>51000</v>
       </c>
-      <c r="J35" s="16"/>
-      <c r="K35" s="28" t="s">
+      <c r="K35" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="L35" s="29">
+      <c r="L35" s="25">
         <f>COUNTIF(DATA!$G$17:$G$26,G17)</f>
         <v>5</v>
       </c>
-      <c r="M35" s="16"/>
-      <c r="N35" s="28" t="s">
+      <c r="N35" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="O35" s="33">
+      <c r="O35" s="29">
         <f ca="1">MIN(DATA!$I$35:$I$37)</f>
         <v>15000</v>
       </c>
-      <c r="P35" s="29" t="str">
+      <c r="P35" s="25" t="str">
         <f ca="1">_xlfn.XLOOKUP(O35,$G$35:$G$37,DATA!$H$35:$H$37)</f>
         <v>Oil</v>
       </c>
-      <c r="Q35" s="16"/>
-      <c r="R35" s="16"/>
-      <c r="S35" s="16"/>
-      <c r="T35" s="16"/>
-      <c r="U35" s="16"/>
-    </row>
-    <row r="36" spans="2:21" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G36">
         <v>24000</v>
       </c>
-      <c r="H36" s="30" t="s">
+      <c r="H36" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="I36" s="31">
+      <c r="I36" s="27">
         <f ca="1">SUMIF(DATA!$C$17:$E$26,C18,DATA!$E$17:$E$26)</f>
         <v>24000</v>
       </c>
@@ -1794,7 +1562,7 @@
         <v>Tyre</v>
       </c>
     </row>
-    <row r="37" spans="2:21" x14ac:dyDescent="0.3">
+    <row r="37" spans="7:16" x14ac:dyDescent="0.3">
       <c r="G37">
         <v>15000</v>
       </c>
@@ -1806,55 +1574,55 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="38" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="N38" s="11" t="s">
+    <row r="38" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="N38" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="O38" s="11"/>
-      <c r="P38" s="11"/>
-    </row>
-    <row r="39" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="G39" s="11" t="s">
+      <c r="O38" s="36"/>
+      <c r="P38" s="36"/>
+    </row>
+    <row r="39" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="G39" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="11"/>
-      <c r="K39" s="11" t="s">
+      <c r="H39" s="36"/>
+      <c r="I39" s="36"/>
+      <c r="J39" s="36"/>
+      <c r="K39" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="L39" s="11"/>
-      <c r="N39" s="11" t="s">
+      <c r="L39" s="36"/>
+      <c r="N39" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="O39" s="11"/>
-      <c r="P39" s="11"/>
-    </row>
-    <row r="40" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="N40" s="11" t="s">
+      <c r="O39" s="36"/>
+      <c r="P39" s="36"/>
+    </row>
+    <row r="40" spans="7:16" x14ac:dyDescent="0.3">
+      <c r="N40" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="O40" s="11"/>
-      <c r="P40" s="11"/>
+      <c r="O40" s="36"/>
+      <c r="P40" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="N38:P38"/>
+    <mergeCell ref="K32:L33"/>
+    <mergeCell ref="N32:P32"/>
+    <mergeCell ref="N39:P39"/>
+    <mergeCell ref="N40:P40"/>
     <mergeCell ref="G11:K11"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="G39:J39"/>
     <mergeCell ref="K39:L39"/>
-    <mergeCell ref="N38:P38"/>
-    <mergeCell ref="K32:L33"/>
-    <mergeCell ref="N32:P32"/>
-    <mergeCell ref="N39:P39"/>
-    <mergeCell ref="N40:P40"/>
     <mergeCell ref="H18:I20"/>
     <mergeCell ref="H32:I33"/>
   </mergeCells>
   <conditionalFormatting sqref="Z15:Z24">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" priority="1">
       <formula>$Z$15=HIGH</formula>
     </cfRule>
     <cfRule type="iconSet" priority="2">

</xml_diff>